<commit_message>
update IC stock , monitor stock
</commit_message>
<xml_diff>
--- a/active.xlsx
+++ b/active.xlsx
@@ -5,22 +5,33 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuhe/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liuhe/PycharmProjects/YJCX_AI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{361F2E79-0D8E-3C46-AECE-9007C5C04E3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B9EBD7-0FA3-6042-B842-96ED3F3D75B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6040" yWindow="500" windowWidth="30240" windowHeight="17760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="上海">#REF!</definedName>
     <definedName name="深圳">#REF!</definedName>
     <definedName name="市">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -365,7 +376,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4510ED14-00A7-AC42-9037-C58A707E96DE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <sheetData/>

</xml_diff>